<commit_message>
Mejora UI y corrección de bugs
</commit_message>
<xml_diff>
--- a/ClientesSolo_INTERIOR.xlsx
+++ b/ClientesSolo_INTERIOR.xlsx
@@ -21051,7 +21051,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -21260,6 +21260,7 @@
     <xf borderId="31" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="31" fillId="0" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="34" fillId="0" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="21" fillId="0" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
@@ -78176,6 +78177,8 @@
       <c r="Q1035" s="84"/>
       <c r="R1035" s="84"/>
       <c r="S1035" s="84"/>
+      <c r="T1035" s="90"/>
+      <c r="U1035" s="90"/>
     </row>
     <row r="1036" ht="15.0" customHeight="1">
       <c r="A1036" s="84"/>
@@ -78197,6 +78200,8 @@
       <c r="Q1036" s="84"/>
       <c r="R1036" s="84"/>
       <c r="S1036" s="84"/>
+      <c r="T1036" s="90"/>
+      <c r="U1036" s="90"/>
     </row>
     <row r="1037" ht="15.0" customHeight="1">
       <c r="A1037" s="84"/>
@@ -78218,6 +78223,8 @@
       <c r="Q1037" s="84"/>
       <c r="R1037" s="84"/>
       <c r="S1037" s="84"/>
+      <c r="T1037" s="90"/>
+      <c r="U1037" s="90"/>
     </row>
     <row r="1038" ht="15.0" customHeight="1">
       <c r="A1038" s="84"/>
@@ -78239,6 +78246,8 @@
       <c r="Q1038" s="84"/>
       <c r="R1038" s="84"/>
       <c r="S1038" s="84"/>
+      <c r="T1038" s="90"/>
+      <c r="U1038" s="90"/>
     </row>
     <row r="1039" ht="15.0" customHeight="1">
       <c r="A1039" s="84"/>
@@ -78260,6 +78269,8 @@
       <c r="Q1039" s="84"/>
       <c r="R1039" s="84"/>
       <c r="S1039" s="84"/>
+      <c r="T1039" s="90"/>
+      <c r="U1039" s="90"/>
     </row>
     <row r="1040" ht="15.0" customHeight="1">
       <c r="A1040" s="84"/>
@@ -78281,6 +78292,8 @@
       <c r="Q1040" s="84"/>
       <c r="R1040" s="84"/>
       <c r="S1040" s="84"/>
+      <c r="T1040" s="90"/>
+      <c r="U1040" s="90"/>
     </row>
     <row r="1041" ht="15.0" customHeight="1">
       <c r="A1041" s="84"/>
@@ -78302,6 +78315,8 @@
       <c r="Q1041" s="84"/>
       <c r="R1041" s="84"/>
       <c r="S1041" s="84"/>
+      <c r="T1041" s="90"/>
+      <c r="U1041" s="90"/>
     </row>
     <row r="1042" ht="15.0" customHeight="1">
       <c r="A1042" s="84"/>
@@ -78323,6 +78338,8 @@
       <c r="Q1042" s="84"/>
       <c r="R1042" s="84"/>
       <c r="S1042" s="84"/>
+      <c r="T1042" s="90"/>
+      <c r="U1042" s="90"/>
     </row>
     <row r="1043" ht="15.0" customHeight="1">
       <c r="A1043" s="84"/>
@@ -78344,6 +78361,8 @@
       <c r="Q1043" s="84"/>
       <c r="R1043" s="84"/>
       <c r="S1043" s="84"/>
+      <c r="T1043" s="90"/>
+      <c r="U1043" s="90"/>
     </row>
     <row r="1044" ht="15.0" customHeight="1">
       <c r="A1044" s="84"/>
@@ -78365,6 +78384,8 @@
       <c r="Q1044" s="84"/>
       <c r="R1044" s="84"/>
       <c r="S1044" s="84"/>
+      <c r="T1044" s="90"/>
+      <c r="U1044" s="90"/>
     </row>
     <row r="1045" ht="15.0" customHeight="1">
       <c r="A1045" s="84"/>
@@ -78386,6 +78407,8 @@
       <c r="Q1045" s="84"/>
       <c r="R1045" s="84"/>
       <c r="S1045" s="84"/>
+      <c r="T1045" s="90"/>
+      <c r="U1045" s="90"/>
     </row>
     <row r="1046" ht="15.0" customHeight="1">
       <c r="A1046" s="84"/>
@@ -78407,6 +78430,8 @@
       <c r="Q1046" s="84"/>
       <c r="R1046" s="84"/>
       <c r="S1046" s="84"/>
+      <c r="T1046" s="90"/>
+      <c r="U1046" s="90"/>
     </row>
     <row r="1047" ht="15.0" customHeight="1">
       <c r="A1047" s="84"/>
@@ -78428,6 +78453,8 @@
       <c r="Q1047" s="84"/>
       <c r="R1047" s="84"/>
       <c r="S1047" s="84"/>
+      <c r="T1047" s="90"/>
+      <c r="U1047" s="90"/>
     </row>
     <row r="1048" ht="15.0" customHeight="1">
       <c r="A1048" s="84"/>
@@ -78449,6 +78476,8 @@
       <c r="Q1048" s="84"/>
       <c r="R1048" s="84"/>
       <c r="S1048" s="84"/>
+      <c r="T1048" s="90"/>
+      <c r="U1048" s="90"/>
     </row>
     <row r="1049" ht="15.0" customHeight="1">
       <c r="A1049" s="84"/>
@@ -78470,6 +78499,8 @@
       <c r="Q1049" s="84"/>
       <c r="R1049" s="84"/>
       <c r="S1049" s="84"/>
+      <c r="T1049" s="90"/>
+      <c r="U1049" s="90"/>
     </row>
     <row r="1050" ht="15.0" customHeight="1">
       <c r="A1050" s="84"/>
@@ -78491,6 +78522,8 @@
       <c r="Q1050" s="84"/>
       <c r="R1050" s="84"/>
       <c r="S1050" s="84"/>
+      <c r="T1050" s="90"/>
+      <c r="U1050" s="90"/>
     </row>
     <row r="1051" ht="15.0" customHeight="1">
       <c r="A1051" s="84"/>
@@ -78512,6 +78545,8 @@
       <c r="Q1051" s="84"/>
       <c r="R1051" s="84"/>
       <c r="S1051" s="84"/>
+      <c r="T1051" s="90"/>
+      <c r="U1051" s="90"/>
     </row>
     <row r="1052" ht="15.0" customHeight="1">
       <c r="A1052" s="84"/>
@@ -78533,6 +78568,8 @@
       <c r="Q1052" s="84"/>
       <c r="R1052" s="84"/>
       <c r="S1052" s="84"/>
+      <c r="T1052" s="90"/>
+      <c r="U1052" s="90"/>
     </row>
     <row r="1053" ht="15.0" customHeight="1">
       <c r="A1053" s="84"/>
@@ -78554,6 +78591,8 @@
       <c r="Q1053" s="84"/>
       <c r="R1053" s="84"/>
       <c r="S1053" s="84"/>
+      <c r="T1053" s="90"/>
+      <c r="U1053" s="90"/>
     </row>
     <row r="1054" ht="15.0" customHeight="1">
       <c r="A1054" s="84"/>
@@ -78575,6 +78614,8 @@
       <c r="Q1054" s="84"/>
       <c r="R1054" s="84"/>
       <c r="S1054" s="84"/>
+      <c r="T1054" s="90"/>
+      <c r="U1054" s="90"/>
     </row>
     <row r="1055" ht="15.0" customHeight="1">
       <c r="A1055" s="84"/>
@@ -78596,6 +78637,8 @@
       <c r="Q1055" s="84"/>
       <c r="R1055" s="84"/>
       <c r="S1055" s="84"/>
+      <c r="T1055" s="90"/>
+      <c r="U1055" s="90"/>
     </row>
     <row r="1056" ht="15.0" customHeight="1">
       <c r="A1056" s="84"/>
@@ -78617,6 +78660,8 @@
       <c r="Q1056" s="84"/>
       <c r="R1056" s="84"/>
       <c r="S1056" s="84"/>
+      <c r="T1056" s="90"/>
+      <c r="U1056" s="90"/>
     </row>
     <row r="1057" ht="15.0" customHeight="1">
       <c r="A1057" s="84"/>
@@ -78638,6 +78683,8 @@
       <c r="Q1057" s="84"/>
       <c r="R1057" s="84"/>
       <c r="S1057" s="84"/>
+      <c r="T1057" s="90"/>
+      <c r="U1057" s="90"/>
     </row>
     <row r="1058" ht="15.0" customHeight="1">
       <c r="A1058" s="84"/>
@@ -78659,6 +78706,8 @@
       <c r="Q1058" s="84"/>
       <c r="R1058" s="84"/>
       <c r="S1058" s="84"/>
+      <c r="T1058" s="90"/>
+      <c r="U1058" s="90"/>
     </row>
     <row r="1059" ht="15.0" customHeight="1">
       <c r="A1059" s="84"/>
@@ -78666,7 +78715,7 @@
       <c r="C1059" s="85"/>
       <c r="D1059" s="85"/>
       <c r="E1059" s="85"/>
-      <c r="F1059" s="90"/>
+      <c r="F1059" s="91"/>
       <c r="G1059" s="87"/>
       <c r="H1059" s="88"/>
       <c r="I1059" s="88"/>
@@ -78680,6 +78729,8 @@
       <c r="Q1059" s="84"/>
       <c r="R1059" s="84"/>
       <c r="S1059" s="84"/>
+      <c r="T1059" s="90"/>
+      <c r="U1059" s="90"/>
     </row>
     <row r="1060" ht="15.0" customHeight="1">
       <c r="A1060" s="84"/>
@@ -78687,7 +78738,7 @@
       <c r="C1060" s="84"/>
       <c r="D1060" s="84"/>
       <c r="E1060" s="84"/>
-      <c r="F1060" s="91"/>
+      <c r="F1060" s="92"/>
       <c r="G1060" s="84"/>
       <c r="H1060" s="84"/>
       <c r="I1060" s="84"/>
@@ -78701,6 +78752,8 @@
       <c r="Q1060" s="84"/>
       <c r="R1060" s="84"/>
       <c r="S1060" s="84"/>
+      <c r="T1060" s="90"/>
+      <c r="U1060" s="90"/>
     </row>
     <row r="1061" ht="15.0" customHeight="1"/>
     <row r="1062" ht="15.0" customHeight="1"/>

</xml_diff>